<commit_message>
Add marketing data for analysis
</commit_message>
<xml_diff>
--- a/data/supplier_scorings/suppliers_list/dev_supplier_list_product_id_3_27-07-2026.xlsx
+++ b/data/supplier_scorings/suppliers_list/dev_supplier_list_product_id_3_27-07-2026.xlsx
@@ -260,8 +260,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -269,15 +273,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -407,511 +403,511 @@
   <dimension ref="A1:U12"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="19.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="21.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="16.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="14.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="22.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="0" width="27.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="21.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="48.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="19.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="21.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="16.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="13.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="14.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="22.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="1" width="27.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="21.19"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1"/>
+      <c r="U1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>3000</v>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="D2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="0" t="n">
+      <c r="F2" s="1" t="n">
         <v>1.3</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="O2" s="0" t="n">
+      <c r="G2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O2" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="P2" s="0" t="n">
+      <c r="P2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T2" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>3001</v>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="B3" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="D3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" s="0" t="n">
+      <c r="F3" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="O3" s="0" t="n">
+      <c r="O3" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="P3" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="T3" s="4" t="s">
+      <c r="P3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T3" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3002</v>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="B4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="3" t="s">
+      <c r="D4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="0" t="n">
+      <c r="F4" s="1" t="n">
         <v>1.12</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" s="0" t="n">
+      <c r="G4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="P4" s="0" t="n">
+      <c r="P4" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="T4" s="4" t="s">
+      <c r="T4" s="3" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>3003</v>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="3" t="s">
+      <c r="D5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="0" t="n">
+      <c r="F5" s="1" t="n">
         <v>0.99</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" s="0" t="n">
+      <c r="G5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="O5" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="P5" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="T5" s="4" t="s">
+      <c r="O5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T5" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>3004</v>
       </c>
-      <c r="B6" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" s="0" t="s">
+      <c r="B6" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="0" t="s">
+      <c r="D6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F6" s="0" t="n">
+      <c r="F6" s="1" t="n">
         <v>1.4</v>
       </c>
-      <c r="G6" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="0" t="n">
+      <c r="G6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="1" t="n">
         <v>350</v>
       </c>
-      <c r="M6" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="O6" s="0" t="n">
+      <c r="M6" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O6" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="P6" s="0" t="n">
+      <c r="P6" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="T6" s="4" t="s">
+      <c r="T6" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>3005</v>
       </c>
-      <c r="B7" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C7" s="0" t="s">
+      <c r="B7" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="0" t="s">
+      <c r="D7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="0" t="n">
+      <c r="F7" s="1" t="n">
         <v>0.84</v>
       </c>
-      <c r="G7" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="O7" s="0" t="n">
+      <c r="G7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="P7" s="0" t="n">
+      <c r="P7" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="T7" s="4" t="s">
+      <c r="T7" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>3006</v>
       </c>
-      <c r="B8" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C8" s="0" t="s">
+      <c r="B8" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" s="0" t="s">
+      <c r="D8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F8" s="0" t="n">
+      <c r="F8" s="1" t="n">
         <v>1.3</v>
       </c>
-      <c r="G8" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" s="0" t="n">
+      <c r="G8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="I8" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="O8" s="0" t="n">
+      <c r="I8" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" s="1" t="n">
         <v>1000</v>
       </c>
-      <c r="P8" s="0" t="n">
+      <c r="P8" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="T8" s="4" t="s">
+      <c r="T8" s="3" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>3007</v>
       </c>
-      <c r="B9" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C9" s="0" t="s">
+      <c r="B9" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="0" t="s">
+      <c r="D9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F9" s="0" t="n">
+      <c r="F9" s="1" t="n">
         <v>1.45</v>
       </c>
-      <c r="G9" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="H9" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="M9" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="O9" s="0" t="n">
+      <c r="G9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="P9" s="0" t="n">
+      <c r="P9" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="T9" s="4" t="s">
+      <c r="T9" s="3" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>3008</v>
       </c>
-      <c r="B10" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" s="0" t="s">
+      <c r="B10" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="E10" s="0" t="s">
+      <c r="D10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F10" s="0" t="n">
+      <c r="F10" s="1" t="n">
         <v>1.46</v>
       </c>
-      <c r="G10" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="0" t="n">
+      <c r="G10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="P10" s="0" t="n">
+      <c r="P10" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="T10" s="4" t="s">
+      <c r="T10" s="3" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>3009</v>
       </c>
-      <c r="B11" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C11" s="0" t="s">
+      <c r="B11" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" s="0" t="s">
+      <c r="D11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F11" s="0" t="n">
+      <c r="F11" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="G11" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="H11" s="0" t="n">
+      <c r="G11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I11" s="0" t="n">
+      <c r="I11" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="O11" s="0" t="n">
+      <c r="O11" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="P11" s="0" t="n">
+      <c r="P11" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="T11" s="4" t="s">
+      <c r="T11" s="3" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>3010</v>
       </c>
-      <c r="B12" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C12" s="0" t="s">
+      <c r="B12" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="0" t="s">
+      <c r="D12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F12" s="0" t="n">
+      <c r="F12" s="1" t="n">
         <v>2.96</v>
       </c>
-      <c r="G12" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="H12" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" s="0" t="n">
+      <c r="G12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="J12" s="0" t="n">
+      <c r="J12" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="O12" s="0" t="n">
+      <c r="O12" s="1" t="n">
         <v>36</v>
       </c>
-      <c r="P12" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" s="4" t="s">
+      <c r="P12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T12" s="3" t="s">
         <v>52</v>
       </c>
     </row>

</xml_diff>